<commit_message>
Save local demand data and script updates
</commit_message>
<xml_diff>
--- a/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
+++ b/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\Demand\InputData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DWRAT_DataScraping\Demand\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E5273E-3D15-4BC9-B0FB-056661624332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB248E3-906D-433F-A207-F6DED776A399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8961FACC-9C35-4F39-BB8E-E3D4A8B78A2C}"/>
+    <workbookView xWindow="5400" yWindow="2370" windowWidth="28800" windowHeight="11295" xr2:uid="{8961FACC-9C35-4F39-BB8E-E3D4A8B78A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Main_Sheet" sheetId="1" r:id="rId1"/>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="178">
   <si>
     <t>Info</t>
   </si>
@@ -707,6 +707,20 @@
   </si>
   <si>
     <t>Required for "POD_StreamStats_Analysis.R". The script uses a single point to represent the exit location of the watershed's main tributary. The watershed boundary layer is required to identify this exit point. (Please consult the documentation for more information)</t>
+  </si>
+  <si>
+    <t>SLO_Pismo</t>
+  </si>
+  <si>
+    <t>SLO</t>
+  </si>
+  <si>
+    <t>C:\Users\PHoupt\Water Boards\Supply and Demand Assessment - Documents\
+Program Watersheds\1. Watershed Folders\SLO &amp; Pismo Creeks\Data\GIS\
+Slo_Pismo_Boundary.gdb</t>
+  </si>
+  <si>
+    <t>DissolvedFeatures</t>
   </si>
 </sst>
 </file>
@@ -844,7 +858,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -893,6 +907,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1504,122 +1521,122 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24A2F77B-58D1-4171-AA16-A7B2F203ADC2}">
   <dimension ref="A1:AX16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" customWidth="1"/>
-    <col min="5" max="5" width="61.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="35.85546875" customWidth="1"/>
+    <col min="5" max="5" width="61.5703125" style="2" customWidth="1"/>
     <col min="6" max="6" width="58" style="12" customWidth="1"/>
-    <col min="7" max="7" width="45.44140625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="40" style="12" customWidth="1"/>
+    <col min="7" max="7" width="45.42578125" style="12" customWidth="1"/>
+    <col min="8" max="8" width="44.85546875" style="12" customWidth="1"/>
     <col min="9" max="9" width="58" style="12" customWidth="1"/>
     <col min="10" max="10" width="58" style="2" customWidth="1"/>
     <col min="11" max="11" width="58" style="15" customWidth="1"/>
     <col min="12" max="12" width="58" style="2" customWidth="1"/>
     <col min="13" max="13" width="52" customWidth="1"/>
     <col min="14" max="14" width="57" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="60.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="91.5546875" customWidth="1"/>
+    <col min="15" max="15" width="60.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="91.5703125" customWidth="1"/>
     <col min="17" max="17" width="52" customWidth="1"/>
-    <col min="18" max="18" width="63.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="90.5546875" customWidth="1"/>
-    <col min="20" max="20" width="53.44140625" customWidth="1"/>
+    <col min="18" max="18" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="90.5703125" customWidth="1"/>
+    <col min="20" max="20" width="53.42578125" customWidth="1"/>
     <col min="21" max="21" width="70" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="136.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="63.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="57.44140625" customWidth="1"/>
-    <col min="25" max="25" width="112.44140625" customWidth="1"/>
-    <col min="26" max="26" width="48.5546875" style="2" customWidth="1"/>
-    <col min="27" max="27" width="85.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="51.5546875" style="2" customWidth="1"/>
-    <col min="29" max="29" width="48.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="65.5546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="94.5546875" customWidth="1"/>
-    <col min="32" max="33" width="65.5546875" customWidth="1"/>
+    <col min="22" max="22" width="136.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="57.42578125" customWidth="1"/>
+    <col min="25" max="25" width="112.42578125" customWidth="1"/>
+    <col min="26" max="26" width="48.5703125" style="2" customWidth="1"/>
+    <col min="27" max="27" width="85.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="51.5703125" style="2" customWidth="1"/>
+    <col min="29" max="29" width="48.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="65.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="94.5703125" customWidth="1"/>
+    <col min="32" max="33" width="65.5703125" customWidth="1"/>
     <col min="34" max="34" width="65" customWidth="1"/>
-    <col min="35" max="37" width="65.5546875" customWidth="1"/>
-    <col min="38" max="38" width="43.44140625" customWidth="1"/>
-    <col min="39" max="39" width="39.44140625" customWidth="1"/>
-    <col min="40" max="40" width="46.5546875" customWidth="1"/>
-    <col min="41" max="41" width="37.44140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="53.5546875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="52.44140625" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="47.5546875" hidden="1" customWidth="1"/>
-    <col min="47" max="47" width="49.5546875" hidden="1" customWidth="1"/>
-    <col min="48" max="48" width="62.44140625" customWidth="1"/>
-    <col min="49" max="49" width="42.5546875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="37" width="65.5703125" customWidth="1"/>
+    <col min="38" max="38" width="43.42578125" customWidth="1"/>
+    <col min="39" max="39" width="39.42578125" customWidth="1"/>
+    <col min="40" max="40" width="46.5703125" customWidth="1"/>
+    <col min="41" max="41" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="39.42578125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="53.5703125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="52.42578125" hidden="1" customWidth="1"/>
+    <col min="46" max="46" width="47.5703125" hidden="1" customWidth="1"/>
+    <col min="47" max="47" width="49.5703125" hidden="1" customWidth="1"/>
+    <col min="48" max="48" width="62.42578125" customWidth="1"/>
+    <col min="49" max="49" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="59.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="27" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="30"/>
       <c r="O1" s="22"/>
-      <c r="P1" s="33" t="s">
+      <c r="P1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="34"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="30" t="s">
+      <c r="Q1" s="35"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="32"/>
-      <c r="AE1" s="36" t="s">
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+      <c r="X1" s="32"/>
+      <c r="Y1" s="32"/>
+      <c r="Z1" s="32"/>
+      <c r="AA1" s="32"/>
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="AF1" s="37"/>
-      <c r="AG1" s="38"/>
-      <c r="AH1" s="25" t="s">
+      <c r="AF1" s="38"/>
+      <c r="AG1" s="39"/>
+      <c r="AH1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="AI1" s="26"/>
-      <c r="AJ1" s="26"/>
-      <c r="AK1" s="26"/>
-      <c r="AL1" s="26"/>
-      <c r="AM1" s="26"/>
-      <c r="AN1" s="26"/>
-      <c r="AO1" s="26"/>
-      <c r="AP1" s="26"/>
-      <c r="AQ1" s="26"/>
-      <c r="AR1" s="26"/>
-      <c r="AS1" s="26"/>
-      <c r="AT1" s="26"/>
-      <c r="AU1" s="26"/>
-      <c r="AV1" s="26"/>
-      <c r="AW1" s="26"/>
-      <c r="AX1" s="26"/>
-    </row>
-    <row r="2" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AI1" s="27"/>
+      <c r="AJ1" s="27"/>
+      <c r="AK1" s="27"/>
+      <c r="AL1" s="27"/>
+      <c r="AM1" s="27"/>
+      <c r="AN1" s="27"/>
+      <c r="AO1" s="27"/>
+      <c r="AP1" s="27"/>
+      <c r="AQ1" s="27"/>
+      <c r="AR1" s="27"/>
+      <c r="AS1" s="27"/>
+      <c r="AT1" s="27"/>
+      <c r="AU1" s="27"/>
+      <c r="AV1" s="27"/>
+      <c r="AW1" s="27"/>
+      <c r="AX1" s="27"/>
+    </row>
+    <row r="2" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1771,7 +1788,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:50" s="11" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:50" s="11" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <f t="shared" ref="A3:A4" si="0">ROW(B3) - 2</f>
         <v>1</v>
@@ -1896,7 +1913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:50" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:50" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1952,21 +1969,38 @@
       </c>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:50" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="1"/>
+    <row r="5" spans="1:50" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>175</v>
+      </c>
       <c r="D5" s="1"/>
+      <c r="E5" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="G5" s="12" t="b">
+        <v>1</v>
+      </c>
       <c r="N5" s="1"/>
       <c r="R5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:50" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:50" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="N6" s="1"/>
       <c r="R6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="N7" s="1"/>
@@ -1980,7 +2014,7 @@
       <c r="AF7" s="15"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="8" spans="1:50" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:50" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="J8" s="12"/>
@@ -1989,7 +2023,7 @@
       <c r="AJ8" s="1"/>
       <c r="AN8" s="1"/>
     </row>
-    <row r="9" spans="1:50" ht="55.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:50" ht="55.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="N9" s="1"/>
@@ -1997,7 +2031,7 @@
       <c r="AD9" s="1"/>
       <c r="AN9" s="1"/>
     </row>
-    <row r="10" spans="1:50" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:50" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="N10" s="1"/>
@@ -2006,7 +2040,7 @@
       <c r="AD10" s="1"/>
       <c r="AN10" s="1"/>
     </row>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
       <c r="N11" s="1"/>
@@ -2031,7 +2065,7 @@
       <c r="AN11" s="11"/>
       <c r="AO11" s="11"/>
     </row>
-    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="J12" s="12"/>
@@ -2042,7 +2076,7 @@
       <c r="AD12" s="1"/>
       <c r="AN12" s="1"/>
     </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="J13" s="12"/>
@@ -2055,7 +2089,7 @@
       <c r="AN13" s="1"/>
       <c r="AV13" s="2"/>
     </row>
-    <row r="14" spans="1:50" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:50" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="J14" s="12"/>
@@ -2065,7 +2099,7 @@
       <c r="AF14" s="11"/>
       <c r="AN14" s="1"/>
     </row>
-    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="N15" s="1"/>
@@ -2073,7 +2107,7 @@
       <c r="AD15" s="1"/>
       <c r="AN15" s="1"/>
     </row>
-    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:50" x14ac:dyDescent="0.25">
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="N16" s="1"/>
@@ -2146,14 +2180,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69755CA-4815-49BC-97C9-A62687C98940}">
   <dimension ref="A1:C47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="85.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="76.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="85.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -2164,7 +2198,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
@@ -2175,7 +2209,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
@@ -2186,7 +2220,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -2197,7 +2231,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
@@ -2208,7 +2242,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -2219,7 +2253,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
@@ -2230,7 +2264,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
@@ -2241,7 +2275,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
@@ -2252,7 +2286,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
@@ -2263,7 +2297,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>15</v>
       </c>
@@ -2274,7 +2308,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
@@ -2285,7 +2319,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
@@ -2296,7 +2330,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
@@ -2307,7 +2341,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>19</v>
       </c>
@@ -2318,7 +2352,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
@@ -2329,7 +2363,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>21</v>
       </c>
@@ -2340,7 +2374,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -2351,7 +2385,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>23</v>
       </c>
@@ -2362,7 +2396,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>24</v>
       </c>
@@ -2373,7 +2407,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>25</v>
       </c>
@@ -2384,7 +2418,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>26</v>
       </c>
@@ -2395,7 +2429,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>27</v>
       </c>
@@ -2406,7 +2440,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>28</v>
       </c>
@@ -2417,7 +2451,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
@@ -2428,7 +2462,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>30</v>
       </c>
@@ -2439,7 +2473,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>31</v>
       </c>
@@ -2450,7 +2484,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>32</v>
       </c>
@@ -2461,7 +2495,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>33</v>
       </c>
@@ -2472,7 +2506,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>34</v>
       </c>
@@ -2483,7 +2517,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>35</v>
       </c>
@@ -2494,7 +2528,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>36</v>
       </c>
@@ -2505,7 +2539,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>37</v>
       </c>
@@ -2516,7 +2550,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>38</v>
       </c>
@@ -2527,7 +2561,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -2538,7 +2572,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>40</v>
       </c>
@@ -2549,7 +2583,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -2560,7 +2594,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>42</v>
       </c>
@@ -2571,7 +2605,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
         <v>43</v>
       </c>
@@ -2582,7 +2616,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>44</v>
       </c>
@@ -2593,7 +2627,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>45</v>
       </c>
@@ -2604,7 +2638,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>46</v>
       </c>
@@ -2615,7 +2649,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>47</v>
       </c>
@@ -2626,7 +2660,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>48</v>
       </c>
@@ -2637,7 +2671,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>49</v>
       </c>
@@ -2648,7 +2682,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>50</v>
       </c>
@@ -2659,7 +2693,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>51</v>
       </c>

</xml_diff>